<commit_message>
Fix Excel number formats
</commit_message>
<xml_diff>
--- a/output/summary_formatted.xlsx
+++ b/output/summary_formatted.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SA\Documents\Claude\Cowork\Projects\005 - MF vs Index\output\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09064E35-F0C1-4E33-B5CB-9B68A665DBD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E12DCF2-E201-492D-A297-354429B7DC63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="360" windowWidth="29040" windowHeight="15960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -89,10 +89,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -102,6 +103,13 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -259,10 +267,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -280,13 +290,34 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -298,41 +329,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="8" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="23">
+  <dxfs count="7">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -379,40 +403,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
@@ -428,105 +418,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF92D050"/>
         </patternFill>
       </fill>
     </dxf>
@@ -841,18 +732,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="12"/>
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="18"/>
+      <c r="F1" s="18"/>
+      <c r="G1" s="19"/>
     </row>
     <row r="2" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="8" t="s">
         <v>18</v>
       </c>
       <c r="B2" s="4" t="s">
@@ -864,18 +755,18 @@
       <c r="D2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="20" t="s">
         <v>3</v>
       </c>
       <c r="F2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="9" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="10" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="6">
@@ -884,21 +775,21 @@
       <c r="C3" s="6">
         <v>0.14467285996769741</v>
       </c>
-      <c r="D3" s="6">
+      <c r="D3" s="21">
         <v>0.92509551473301777</v>
       </c>
       <c r="E3" s="6">
         <v>-0.15368025852407979</v>
       </c>
-      <c r="F3" s="7">
+      <c r="F3" s="24">
         <v>1</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="11" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="10" t="s">
         <v>8</v>
       </c>
       <c r="B4" s="6">
@@ -907,21 +798,21 @@
       <c r="C4" s="6">
         <v>0.1420669303142994</v>
       </c>
-      <c r="D4" s="6">
+      <c r="D4" s="21">
         <v>0.73813152230784695</v>
       </c>
       <c r="E4" s="6">
         <v>-0.16364563899031101</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="24">
         <v>1</v>
       </c>
-      <c r="G4" s="16" t="s">
+      <c r="G4" s="11" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="10" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="6">
@@ -930,21 +821,21 @@
       <c r="C5" s="6">
         <v>0.13245577380712489</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="21">
         <v>0.78455035843446741</v>
       </c>
       <c r="E5" s="6">
         <v>-0.1539325842696628</v>
       </c>
-      <c r="F5" s="7">
+      <c r="F5" s="24">
         <v>1</v>
       </c>
-      <c r="G5" s="16" t="s">
+      <c r="G5" s="11" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="10" t="s">
         <v>10</v>
       </c>
       <c r="B6" s="6">
@@ -953,21 +844,21 @@
       <c r="C6" s="6">
         <v>0.1362273774781462</v>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="21">
         <v>0.66338807676703149</v>
       </c>
       <c r="E6" s="6">
         <v>-0.16382705516343929</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F6" s="24">
         <v>0.97397260273972608</v>
       </c>
-      <c r="G6" s="16" t="s">
+      <c r="G6" s="11" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="10" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="6">
@@ -976,21 +867,21 @@
       <c r="C7" s="6">
         <v>0.13658479408102239</v>
       </c>
-      <c r="D7" s="6">
+      <c r="D7" s="21">
         <v>0.63569622003248805</v>
       </c>
       <c r="E7" s="6">
         <v>-0.1735485660449155</v>
       </c>
-      <c r="F7" s="7">
+      <c r="F7" s="24">
         <v>1</v>
       </c>
-      <c r="G7" s="16" t="s">
+      <c r="G7" s="11" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="15" t="s">
+      <c r="A8" s="10" t="s">
         <v>12</v>
       </c>
       <c r="B8" s="6">
@@ -999,21 +890,21 @@
       <c r="C8" s="6">
         <v>0.13576666508747609</v>
       </c>
-      <c r="D8" s="6">
+      <c r="D8" s="21">
         <v>0.60840033654486736</v>
       </c>
       <c r="E8" s="6">
         <v>-0.17344398340248959</v>
       </c>
-      <c r="F8" s="7">
+      <c r="F8" s="24">
         <v>0.98630136986301364</v>
       </c>
-      <c r="G8" s="16" t="s">
+      <c r="G8" s="11" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="10" t="s">
         <v>13</v>
       </c>
       <c r="B9" s="6">
@@ -1022,62 +913,62 @@
       <c r="C9" s="6">
         <v>0.1375893072204174</v>
       </c>
-      <c r="D9" s="6">
+      <c r="D9" s="21">
         <v>0.52398250327576978</v>
       </c>
       <c r="E9" s="6">
         <v>-0.1743660267341437</v>
       </c>
-      <c r="F9" s="7">
+      <c r="F9" s="24">
         <v>0.55205479452054795</v>
       </c>
-      <c r="G9" s="16" t="s">
+      <c r="G9" s="11" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="8">
+      <c r="B10" s="7">
         <v>0.13166670395439589</v>
       </c>
-      <c r="C10" s="8">
+      <c r="C10" s="7">
         <v>0.14144895088687759</v>
       </c>
-      <c r="D10" s="8">
+      <c r="D10" s="22">
         <v>0.47131282018282339</v>
       </c>
-      <c r="E10" s="8">
+      <c r="E10" s="7">
         <v>-0.1656191568910286</v>
       </c>
-      <c r="F10" s="9" t="s">
+      <c r="F10" s="25" t="s">
         <v>19</v>
       </c>
-      <c r="G10" s="18" t="s">
+      <c r="G10" s="13" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="20">
+      <c r="B11" s="15">
         <v>0.1173799693784383</v>
       </c>
-      <c r="C11" s="20">
+      <c r="C11" s="15">
         <v>0.1355276147653644</v>
       </c>
-      <c r="D11" s="20">
+      <c r="D11" s="23">
         <v>0.38648927356334323</v>
       </c>
-      <c r="E11" s="20">
+      <c r="E11" s="15">
         <v>-0.21623113728376889</v>
       </c>
-      <c r="F11" s="21">
+      <c r="F11" s="26">
         <v>0.22602739726027399</v>
       </c>
-      <c r="G11" s="22" t="s">
+      <c r="G11" s="16" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1085,27 +976,6 @@
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="A16">
-    <cfRule type="containsText" dxfId="4" priority="7" operator="containsText" text="Yes">
-      <formula>NOT(ISERROR(SEARCH("Yes",A16)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G1048576">
-    <cfRule type="containsText" dxfId="3" priority="5" operator="containsText" text="No">
-      <formula>NOT(ISERROR(SEARCH("No",G2)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="6" operator="containsText" text="Yes">
-      <formula>NOT(ISERROR(SEARCH("Yes",G2)))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G3:G11">
-    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
-      <formula>"No"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
-      <formula>"Yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="D3:D11">
     <cfRule type="colorScale" priority="2">
       <colorScale>
@@ -1130,6 +1000,14 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="G3:G11">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
+      <formula>"No"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
+      <formula>"Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">

</xml_diff>